<commit_message>
feat: varredura e atualizacao com dias 16 e 17/10 avancando semana para 12 a 17 e 46 lojas resgatadas
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-09).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-09).xlsx
@@ -938,31 +938,31 @@
     <t>215</t>
   </si>
   <si>
-    <t>30</t>
+    <t>29</t>
   </si>
   <si>
-    <t>R$ 8.877,51</t>
+    <t>R$ 8.923,57</t>
   </si>
   <si>
-    <t>94.9</t>
+    <t>95.3</t>
   </si>
   <si>
     <t>63.6</t>
   </si>
   <si>
-    <t>6.19</t>
+    <t>6.24</t>
   </si>
   <si>
-    <t>22.4</t>
+    <t>22.5</t>
   </si>
   <si>
-    <t>10.0</t>
+    <t>10.1</t>
   </si>
   <si>
     <t>6.3</t>
   </si>
   <si>
-    <t>30.0%</t>
+    <t>30.1%</t>
   </si>
   <si>
     <t>18.2%</t>
@@ -25192,7 +25192,7 @@
         <v>19863</v>
       </c>
       <c r="B159" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C159" s="4">
         <v>51</v>
@@ -25222,18 +25222,30 @@
         <v>58</v>
       </c>
       <c r="L159" s="4"/>
-      <c r="M159" s="5"/>
-      <c r="N159" s="6"/>
+      <c r="M159" s="5">
+        <v>17444.720000000001</v>
+      </c>
+      <c r="N159" s="6">
+        <v>173</v>
+      </c>
       <c r="O159" s="6">
         <v>143</v>
       </c>
-      <c r="P159" s="7"/>
-      <c r="Q159" s="8"/>
-      <c r="R159" s="8"/>
+      <c r="P159" s="7">
+        <v>16.396666470588237</v>
+      </c>
+      <c r="Q159" s="8">
+        <v>36.05492957746479</v>
+      </c>
+      <c r="R159" s="8">
+        <v>11.122262142857144</v>
+      </c>
       <c r="S159" s="8">
         <v>7</v>
       </c>
-      <c r="T159" s="9"/>
+      <c r="T159" s="9">
+        <v>0.09154929577464789</v>
+      </c>
       <c r="U159" s="9">
         <v>0.083916083916083919</v>
       </c>

</xml_diff>